<commit_message>
added the new version of school discipline action removing the unmatched stratification Labels
</commit_message>
<xml_diff>
--- a/statewide_data.xlsx
+++ b/statewide_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,7 +480,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>82092</t>
+          <t>73067</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>836</t>
+          <t>428</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>33775</t>
+          <t>32209</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>61087</t>
+          <t>57058</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4629</t>
+          <t>3309</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>77440</t>
+          <t>69758</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>28073</t>
+          <t>22807</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13270</t>
+          <t>9933</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>193</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1391</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>53976</t>
+          <t>50260</t>
         </is>
       </c>
     </row>
@@ -801,22 +801,22 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Migrant Status</t>
+          <t>Economic Status</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Migrant</t>
+          <t>Not Econ Disadv</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MIG1</t>
+          <t>NOT3</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>16009</t>
         </is>
       </c>
     </row>
@@ -829,22 +829,22 @@
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>Race/Ethnicity</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Non-binary</t>
+          <t>Amer Indian</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>NON10</t>
+          <t>P</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>1305</t>
         </is>
       </c>
     </row>
@@ -857,22 +857,22 @@
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Economic Status</t>
+          <t>Race/Ethnicity</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Not Econ Disadv</t>
+          <t>Pacific Isle</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>NOT3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>20982</t>
+          <t>33</t>
         </is>
       </c>
     </row>
@@ -885,22 +885,22 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Migrant Status</t>
+          <t>Grade Level</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Not Migrant</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>NOT4</t>
+          <t>PK1</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>82079</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -918,17 +918,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Amer Indian</t>
+          <t>Two or More</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1555</t>
+          <t>4800</t>
         </is>
       </c>
     </row>
@@ -941,22 +941,22 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Race/Ethnicity</t>
+          <t>Disability Status</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pacific Isle</t>
+          <t>SwD</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>SWD1</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>28020</t>
         </is>
       </c>
     </row>
@@ -969,22 +969,22 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Grade Level</t>
+          <t>Disability Status</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>SwoD</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>PK1</t>
+          <t>SWO1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>45047</t>
         </is>
       </c>
     </row>
@@ -997,22 +997,22 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Race/Ethnicity</t>
+          <t>Grade Level</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Two or More</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>UNK8</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>6903</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1025,22 +1025,22 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Disability Status</t>
+          <t>Race/Ethnicity</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>SwD</t>
+          <t>White</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SWD1</t>
+          <t>W</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>28355</t>
+          <t>24359</t>
         </is>
       </c>
     </row>
@@ -1053,22 +1053,22 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Disability Status</t>
+          <t>Grade Level</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SwoD</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SWO1</t>
+          <t>X1012</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>53737</t>
+          <t>8096</t>
         </is>
       </c>
     </row>
@@ -1081,22 +1081,22 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Economic Status</t>
+          <t>Grade Level</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>UNK3</t>
+          <t>X113</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>5351</t>
         </is>
       </c>
     </row>
@@ -1109,22 +1109,22 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>EL Status</t>
+          <t>Grade Level</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>UNK4</t>
+          <t>X1210</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>3388</t>
         </is>
       </c>
     </row>
@@ -1137,22 +1137,22 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Race/Ethnicity</t>
+          <t>Grade Level</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>UNK5</t>
+          <t>X1S2</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2105</t>
         </is>
       </c>
     </row>
@@ -1165,22 +1165,22 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>Grade Level</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>UNK7</t>
+          <t>X2N2</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2555</t>
         </is>
       </c>
     </row>
@@ -1198,17 +1198,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>UNK8</t>
+          <t>X3R2</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3273</t>
         </is>
       </c>
     </row>
@@ -1221,22 +1221,22 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Race/Ethnicity</t>
+          <t>Grade Level</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>X4T2</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>25694</t>
+          <t>4153</t>
         </is>
       </c>
     </row>
@@ -1254,17 +1254,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>X1012</t>
+          <t>X5T3</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>9418</t>
+          <t>4804</t>
         </is>
       </c>
     </row>
@@ -1282,17 +1282,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>X113</t>
+          <t>X6T3</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>6034</t>
+          <t>8327</t>
         </is>
       </c>
     </row>
@@ -1310,17 +1310,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>X1210</t>
+          <t>X7T2</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2944</t>
+          <t>9529</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>X1S2</t>
+          <t>X8T2</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2181</t>
+          <t>9435</t>
         </is>
       </c>
     </row>
@@ -1366,213 +1366,17 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>X2N2</t>
+          <t>X9T3</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2347</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>[Statewide]</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Grade Level</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>X3R2</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>2753</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>[Statewide]</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Grade Level</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>X4T2</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>3357</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>[Statewide]</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Grade Level</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>X5T3</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>4338</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>[Statewide]</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Grade Level</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>X6T3</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>9281</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>[Statewide]</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Grade Level</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>X7T2</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>11511</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>[Statewide]</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Grade Level</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>X8T2</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>12652</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>[Statewide]</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Grade Level</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>X9T3</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>13192</t>
+          <t>10458</t>
         </is>
       </c>
     </row>

</xml_diff>